<commit_message>
updated error on interpolation
</commit_message>
<xml_diff>
--- a/resultsUTM.xlsx
+++ b/resultsUTM.xlsx
@@ -636,7 +636,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>10.53368243087264</v>
+        <v>10.49774981950786</v>
       </c>
       <c r="C2" t="n">
         <v>-66.8894638888889</v>
@@ -645,7 +645,7 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -653,16 +653,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>10.52857664048812</v>
+        <v>10.50203667566391</v>
       </c>
       <c r="C3" t="n">
-        <v>-66.88232409661181</v>
+        <v>-66.88708416257479</v>
       </c>
       <c r="D3" t="n">
         <v>10</v>
       </c>
       <c r="E3" t="n">
-        <v>4.5</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="4">
@@ -670,16 +670,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>10.52253203210929</v>
+        <v>10.50564941049929</v>
       </c>
       <c r="C4" t="n">
-        <v>-66.87696400422162</v>
+        <v>-66.88321428806312</v>
       </c>
       <c r="D4" t="n">
         <v>20</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -1214,16 +1214,16 @@
         <v>34</v>
       </c>
       <c r="B36" t="n">
-        <v>10.51409073659551</v>
+        <v>10.50564941049929</v>
       </c>
       <c r="C36" t="n">
-        <v>-66.89883854618395</v>
+        <v>-66.89571348971469</v>
       </c>
       <c r="D36" t="n">
         <v>340</v>
       </c>
       <c r="E36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
@@ -1231,16 +1231,16 @@
         <v>35</v>
       </c>
       <c r="B37" t="n">
-        <v>10.52415331794662</v>
+        <v>10.50203667566391</v>
       </c>
       <c r="C37" t="n">
-        <v>-66.8958102799791</v>
+        <v>-66.89184361520302</v>
       </c>
       <c r="D37" t="n">
         <v>350</v>
       </c>
       <c r="E37" t="n">
-        <v>4</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="38">
@@ -1248,7 +1248,7 @@
         <v>36</v>
       </c>
       <c r="B38" t="n">
-        <v>10.53368243087264</v>
+        <v>10.49774981950786</v>
       </c>
       <c r="C38" t="n">
         <v>-66.8894638888889</v>
@@ -1257,7 +1257,7 @@
         <v>0</v>
       </c>
       <c r="E38" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -1265,7 +1265,7 @@
         <v>37</v>
       </c>
       <c r="B39" t="n">
-        <v>10.55164873655503</v>
+        <v>10.51571612519025</v>
       </c>
       <c r="C39" t="n">
         <v>-66.8894638888889</v>
@@ -1274,7 +1274,7 @@
         <v>0</v>
       </c>
       <c r="E39" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40">
@@ -1282,16 +1282,16 @@
         <v>38</v>
       </c>
       <c r="B40" t="n">
-        <v>10.54626991090712</v>
+        <v>10.51972999343223</v>
       </c>
       <c r="C40" t="n">
-        <v>-66.87915026407765</v>
+        <v>-66.88391087622782</v>
       </c>
       <c r="D40" t="n">
         <v>10</v>
       </c>
       <c r="E40" t="n">
-        <v>6.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="41">
@@ -1299,16 +1299,16 @@
         <v>39</v>
       </c>
       <c r="B41" t="n">
-        <v>10.53941453128238</v>
+        <v>10.52253203210929</v>
       </c>
       <c r="C41" t="n">
-        <v>-66.87071303617189</v>
+        <v>-66.87696400422162</v>
       </c>
       <c r="D41" t="n">
         <v>20</v>
       </c>
       <c r="E41" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42">
@@ -1843,16 +1843,16 @@
         <v>71</v>
       </c>
       <c r="B73" t="n">
-        <v>10.53097329701385</v>
+        <v>10.52253203210929</v>
       </c>
       <c r="C73" t="n">
-        <v>-66.90508917198048</v>
+        <v>-66.90196377355619</v>
       </c>
       <c r="D73" t="n">
         <v>340</v>
       </c>
       <c r="E73" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="74">
@@ -1860,16 +1860,16 @@
         <v>72</v>
       </c>
       <c r="B74" t="n">
-        <v>10.54184659626623</v>
+        <v>10.51972999343223</v>
       </c>
       <c r="C74" t="n">
-        <v>-66.89898402137779</v>
+        <v>-66.89501690154999</v>
       </c>
       <c r="D74" t="n">
         <v>350</v>
       </c>
       <c r="E74" t="n">
-        <v>6</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="75">
@@ -1877,7 +1877,7 @@
         <v>73</v>
       </c>
       <c r="B75" t="n">
-        <v>10.55164873655503</v>
+        <v>10.51571612519025</v>
       </c>
       <c r="C75" t="n">
         <v>-66.8894638888889</v>
@@ -1886,7 +1886,7 @@
         <v>0</v>
       </c>
       <c r="E75" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1935,10 +1935,10 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1165197.197817992</v>
+        <v>1161221.701781032</v>
       </c>
       <c r="C2" t="n">
-        <v>730966.9535116111</v>
+        <v>730993.6920087057</v>
       </c>
       <c r="D2" t="n">
         <v>19</v>
@@ -1947,7 +1947,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -1955,10 +1955,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1164637.578002534</v>
+        <v>1161697.739867128</v>
       </c>
       <c r="C3" t="n">
-        <v>731752.4497410624</v>
+        <v>731251.070125664</v>
       </c>
       <c r="D3" t="n">
         <v>19</v>
@@ -1967,7 +1967,7 @@
         <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>4.5</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="4">
@@ -1975,10 +1975,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1163972.782121793</v>
+        <v>1162100.297306176</v>
       </c>
       <c r="C4" t="n">
-        <v>732343.8239250184</v>
+        <v>731672.1017393199</v>
       </c>
       <c r="D4" t="n">
         <v>19</v>
@@ -1987,7 +1987,7 @@
         <v>20</v>
       </c>
       <c r="F4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -2615,10 +2615,10 @@
         <v>34</v>
       </c>
       <c r="B36" t="n">
-        <v>1163022.732732167</v>
+        <v>1162091.10133474</v>
       </c>
       <c r="C36" t="n">
-        <v>729955.1277799493</v>
+        <v>730303.5437371819</v>
       </c>
       <c r="D36" t="n">
         <v>19</v>
@@ -2627,7 +2627,7 @@
         <v>340</v>
       </c>
       <c r="F36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
@@ -2635,10 +2635,10 @@
         <v>35</v>
       </c>
       <c r="B37" t="n">
-        <v>1164138.249365305</v>
+        <v>1161694.239370159</v>
       </c>
       <c r="C37" t="n">
-        <v>730279.2193067948</v>
+        <v>730729.9438162486</v>
       </c>
       <c r="D37" t="n">
         <v>19</v>
@@ -2647,7 +2647,7 @@
         <v>350</v>
       </c>
       <c r="F37" t="n">
-        <v>4</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="38">
@@ -2655,10 +2655,10 @@
         <v>36</v>
       </c>
       <c r="B38" t="n">
-        <v>1165197.197817992</v>
+        <v>1161221.701781032</v>
       </c>
       <c r="C38" t="n">
-        <v>730966.9535116111</v>
+        <v>730993.6920087057</v>
       </c>
       <c r="D38" t="n">
         <v>19</v>
@@ -2667,7 +2667,7 @@
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -2675,10 +2675,10 @@
         <v>37</v>
       </c>
       <c r="B39" t="n">
-        <v>1167184.948751044</v>
+        <v>1163209.448829045</v>
       </c>
       <c r="C39" t="n">
-        <v>730953.5503679136</v>
+        <v>730980.3340589586</v>
       </c>
       <c r="D39" t="n">
         <v>19</v>
@@ -2687,7 +2687,7 @@
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40">
@@ -2695,10 +2695,10 @@
         <v>38</v>
       </c>
       <c r="B40" t="n">
-        <v>1166597.482236777</v>
+        <v>1163657.629530344</v>
       </c>
       <c r="C40" t="n">
-        <v>732086.6763928575</v>
+        <v>731585.3284837832</v>
       </c>
       <c r="D40" t="n">
         <v>19</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="F40" t="n">
-        <v>6.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="41">
@@ -2715,10 +2715,10 @@
         <v>39</v>
       </c>
       <c r="B41" t="n">
-        <v>1165845.283475432</v>
+        <v>1163972.782121793</v>
       </c>
       <c r="C41" t="n">
-        <v>733015.5290156588</v>
+        <v>732343.8239250184</v>
       </c>
       <c r="D41" t="n">
         <v>19</v>
@@ -2727,7 +2727,7 @@
         <v>20</v>
       </c>
       <c r="F41" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42">
@@ -3355,10 +3355,10 @@
         <v>71</v>
       </c>
       <c r="B73" t="n">
-        <v>1164885.986000802</v>
+        <v>1163954.360952203</v>
       </c>
       <c r="C73" t="n">
-        <v>729258.2827548694</v>
+        <v>729606.7074503823</v>
       </c>
       <c r="D73" t="n">
         <v>19</v>
@@ -3367,7 +3367,7 @@
         <v>340</v>
       </c>
       <c r="F73" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="74">
@@ -3375,10 +3375,10 @@
         <v>72</v>
       </c>
       <c r="B74" t="n">
-        <v>1166093.450795261</v>
+        <v>1163649.448096665</v>
       </c>
       <c r="C74" t="n">
-        <v>729918.6157167868</v>
+        <v>730369.3668751053</v>
       </c>
       <c r="D74" t="n">
         <v>19</v>
@@ -3387,7 +3387,7 @@
         <v>350</v>
       </c>
       <c r="F74" t="n">
-        <v>6</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="75">
@@ -3395,10 +3395,10 @@
         <v>73</v>
       </c>
       <c r="B75" t="n">
-        <v>1167184.948751044</v>
+        <v>1163209.448829045</v>
       </c>
       <c r="C75" t="n">
-        <v>730953.5503679136</v>
+        <v>730980.3340589586</v>
       </c>
       <c r="D75" t="n">
         <v>19</v>
@@ -3407,7 +3407,7 @@
         <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cambio en seleccion de iconos
</commit_message>
<xml_diff>
--- a/resultsUTM.xlsx
+++ b/resultsUTM.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,27 +513,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1160227.828983885</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>731000.3625090888</v>
+        <v>166021.4430805406</v>
       </c>
       <c r="D2" t="n">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="n">
-        <v>1160395.180980101</v>
-      </c>
-      <c r="C3" t="n">
-        <v>754726.4470557353</v>
-      </c>
-      <c r="D3" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -687,16 +673,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>10.52377437938858</v>
+        <v>10.51210528878385</v>
       </c>
       <c r="C5" t="n">
-        <v>-66.86890599615849</v>
+        <v>-66.87575914482575</v>
       </c>
       <c r="D5" t="n">
         <v>30</v>
       </c>
       <c r="E5" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -704,16 +690,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>10.52317278993719</v>
+        <v>10.50941066445419</v>
       </c>
       <c r="C6" t="n">
-        <v>-66.86009870446183</v>
+        <v>-66.87184556315569</v>
       </c>
       <c r="D6" t="n">
         <v>40</v>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -857,16 +843,16 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>10.47202067151893</v>
+        <v>10.46855582240753</v>
       </c>
       <c r="C15" t="n">
-        <v>-66.86916952834326</v>
+        <v>-66.86497096900254</v>
       </c>
       <c r="D15" t="n">
         <v>130</v>
       </c>
       <c r="E15" t="n">
-        <v>2.9</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="16">
@@ -874,16 +860,16 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>10.47156259440271</v>
+        <v>10.46468077722861</v>
       </c>
       <c r="C16" t="n">
-        <v>-66.87478374641827</v>
+        <v>-66.86891214580925</v>
       </c>
       <c r="D16" t="n">
         <v>140</v>
       </c>
       <c r="E16" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="17">
@@ -925,16 +911,16 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>10.45337988958488</v>
+        <v>10.45780324358407</v>
       </c>
       <c r="C19" t="n">
-        <v>-66.88311894896212</v>
+        <v>-66.88391198727473</v>
       </c>
       <c r="D19" t="n">
         <v>170</v>
       </c>
       <c r="E19" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="20">
@@ -1095,16 +1081,16 @@
         <v>27</v>
       </c>
       <c r="B29" t="n">
-        <v>10.48876653629103</v>
+        <v>10.48876585181897</v>
       </c>
       <c r="C29" t="n">
-        <v>-66.89859969541307</v>
+        <v>-66.91230340516566</v>
       </c>
       <c r="D29" t="n">
         <v>270</v>
       </c>
       <c r="E29" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="30">
@@ -1112,16 +1098,16 @@
         <v>28</v>
       </c>
       <c r="B30" t="n">
-        <v>10.49110624432473</v>
+        <v>10.49266564658427</v>
       </c>
       <c r="C30" t="n">
-        <v>-66.90295951057013</v>
+        <v>-66.91195670506306</v>
       </c>
       <c r="D30" t="n">
         <v>280</v>
       </c>
       <c r="E30" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="31">
@@ -1129,16 +1115,16 @@
         <v>29</v>
       </c>
       <c r="B31" t="n">
-        <v>10.49183897075209</v>
+        <v>10.49798288788125</v>
       </c>
       <c r="C31" t="n">
-        <v>-66.89804882410189</v>
+        <v>-66.91521920606223</v>
       </c>
       <c r="D31" t="n">
         <v>290</v>
       </c>
       <c r="E31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
@@ -1146,16 +1132,16 @@
         <v>30</v>
       </c>
       <c r="B32" t="n">
-        <v>10.49550381123731</v>
+        <v>10.50224051548196</v>
       </c>
       <c r="C32" t="n">
-        <v>-66.90133190810936</v>
+        <v>-66.91320044438086</v>
       </c>
       <c r="D32" t="n">
         <v>300</v>
       </c>
       <c r="E32" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
@@ -1163,16 +1149,16 @@
         <v>31</v>
       </c>
       <c r="B33" t="n">
-        <v>10.49454084948603</v>
+        <v>10.50608875571192</v>
       </c>
       <c r="C33" t="n">
-        <v>-66.89646245331389</v>
+        <v>-66.91046036622406</v>
       </c>
       <c r="D33" t="n">
         <v>310</v>
       </c>
       <c r="E33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34">
@@ -1197,16 +1183,16 @@
         <v>33</v>
       </c>
       <c r="B35" t="n">
-        <v>10.51988469886784</v>
+        <v>10.51210528878385</v>
       </c>
       <c r="C35" t="n">
-        <v>-66.90773734114036</v>
+        <v>-66.90316863295206</v>
       </c>
       <c r="D35" t="n">
         <v>330</v>
       </c>
       <c r="E35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36">
@@ -1316,16 +1302,16 @@
         <v>40</v>
       </c>
       <c r="B42" t="n">
-        <v>10.53933293784263</v>
+        <v>10.52766404355303</v>
       </c>
       <c r="C42" t="n">
-        <v>-66.8597676578074</v>
+        <v>-66.86662149805899</v>
       </c>
       <c r="D42" t="n">
         <v>30</v>
       </c>
       <c r="E42" t="n">
-        <v>6.5</v>
+        <v>5</v>
       </c>
     </row>
     <row r="43">
@@ -1333,16 +1319,16 @@
         <v>41</v>
       </c>
       <c r="B43" t="n">
-        <v>10.53693448293342</v>
+        <v>10.52317278993719</v>
       </c>
       <c r="C43" t="n">
-        <v>-66.84835079749757</v>
+        <v>-66.86009870446183</v>
       </c>
       <c r="D43" t="n">
         <v>40</v>
       </c>
       <c r="E43" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="44">
@@ -1486,16 +1472,16 @@
         <v>50</v>
       </c>
       <c r="B52" t="n">
-        <v>10.46047096074405</v>
+        <v>10.45700592847735</v>
       </c>
       <c r="C52" t="n">
-        <v>-66.85517469536563</v>
+        <v>-66.85097644865398</v>
       </c>
       <c r="D52" t="n">
         <v>130</v>
       </c>
       <c r="E52" t="n">
-        <v>4.9</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="53">
@@ -1503,16 +1489,16 @@
         <v>51</v>
       </c>
       <c r="B53" t="n">
-        <v>10.45779885258807</v>
+        <v>10.45091682055812</v>
       </c>
       <c r="C53" t="n">
-        <v>-66.86304080571429</v>
+        <v>-66.85716972595074</v>
       </c>
       <c r="D53" t="n">
         <v>140</v>
       </c>
       <c r="E53" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="54">
@@ -1554,16 +1540,16 @@
         <v>54</v>
       </c>
       <c r="B56" t="n">
-        <v>10.43568645401288</v>
+        <v>10.44010981584035</v>
       </c>
       <c r="C56" t="n">
-        <v>-66.87994702151873</v>
+        <v>-66.88073996952933</v>
       </c>
       <c r="D56" t="n">
         <v>170</v>
       </c>
       <c r="E56" t="n">
-        <v>6</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="57">
@@ -1724,16 +1710,16 @@
         <v>64</v>
       </c>
       <c r="B66" t="n">
-        <v>10.48876549328599</v>
+        <v>10.4887640265602</v>
       </c>
       <c r="C66" t="n">
-        <v>-66.91687130839983</v>
+        <v>-66.93057501802541</v>
       </c>
       <c r="D66" t="n">
         <v>270</v>
       </c>
       <c r="E66" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="67">
@@ -1741,16 +1727,16 @@
         <v>65</v>
       </c>
       <c r="B67" t="n">
-        <v>10.49422479585263</v>
+        <v>10.49578369208883</v>
       </c>
       <c r="C67" t="n">
-        <v>-66.92095399025365</v>
+        <v>-66.92995136614189</v>
       </c>
       <c r="D67" t="n">
         <v>280</v>
       </c>
       <c r="E67" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="68">
@@ -1758,16 +1744,16 @@
         <v>66</v>
       </c>
       <c r="B68" t="n">
-        <v>10.49798288788125</v>
+        <v>10.50412588313117</v>
       </c>
       <c r="C68" t="n">
-        <v>-66.91521920606223</v>
+        <v>-66.93239027034602</v>
       </c>
       <c r="D68" t="n">
         <v>290</v>
       </c>
       <c r="E68" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="69">
@@ -1775,16 +1761,16 @@
         <v>67</v>
       </c>
       <c r="B69" t="n">
-        <v>10.50448598566001</v>
+        <v>10.5112221023238</v>
       </c>
       <c r="C69" t="n">
-        <v>-66.91715673809496</v>
+        <v>-66.9290259642783</v>
       </c>
       <c r="D69" t="n">
         <v>300</v>
       </c>
       <c r="E69" t="n">
-        <v>3.5</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70">
@@ -1792,16 +1778,16 @@
         <v>68</v>
       </c>
       <c r="B70" t="n">
-        <v>10.50608875571192</v>
+        <v>10.51763604877479</v>
       </c>
       <c r="C70" t="n">
-        <v>-66.91046036622406</v>
+        <v>-66.92445932554698</v>
       </c>
       <c r="D70" t="n">
         <v>310</v>
       </c>
       <c r="E70" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="71">
@@ -1826,16 +1812,16 @@
         <v>70</v>
       </c>
       <c r="B72" t="n">
-        <v>10.53544332278665</v>
+        <v>10.52766404355303</v>
       </c>
       <c r="C72" t="n">
-        <v>-66.91687544887135</v>
+        <v>-66.91230627971881</v>
       </c>
       <c r="D72" t="n">
         <v>330</v>
       </c>
       <c r="E72" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="73">
@@ -1995,10 +1981,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1164116.218326742</v>
+        <v>1162820.076443251</v>
       </c>
       <c r="C5" t="n">
-        <v>733225.1350259718</v>
+        <v>732483.5503219831</v>
       </c>
       <c r="D5" t="n">
         <v>19</v>
@@ -2007,7 +1993,7 @@
         <v>30</v>
       </c>
       <c r="F5" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -2015,10 +2001,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>1164056.226077507</v>
+        <v>1162524.849140179</v>
       </c>
       <c r="C6" t="n">
-        <v>734189.8722406242</v>
+        <v>732914.0708996342</v>
       </c>
       <c r="D6" t="n">
         <v>19</v>
@@ -2027,7 +2013,7 @@
         <v>40</v>
       </c>
       <c r="F6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -2195,10 +2181,10 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>1158390.053822168</v>
+        <v>1158009.818931899</v>
       </c>
       <c r="C15" t="n">
-        <v>733235.099177414</v>
+        <v>733697.4594539634</v>
       </c>
       <c r="D15" t="n">
         <v>19</v>
@@ -2207,7 +2193,7 @@
         <v>130</v>
       </c>
       <c r="F15" t="n">
-        <v>2.9</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="16">
@@ -2215,10 +2201,10 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>1158335.220876137</v>
+        <v>1157578.168469723</v>
       </c>
       <c r="C16" t="n">
-        <v>732620.6580264606</v>
+        <v>733268.7743661823</v>
       </c>
       <c r="D16" t="n">
         <v>19</v>
@@ -2227,7 +2213,7 @@
         <v>140</v>
       </c>
       <c r="F16" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="17">
@@ -2275,10 +2261,10 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>1156317.385136057</v>
+        <v>1156806.191904636</v>
       </c>
       <c r="C19" t="n">
-        <v>731721.4201896497</v>
+        <v>731631.2926654967</v>
       </c>
       <c r="D19" t="n">
         <v>19</v>
@@ -2287,7 +2273,7 @@
         <v>170</v>
       </c>
       <c r="F19" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="20">
@@ -2475,10 +2461,10 @@
         <v>27</v>
       </c>
       <c r="B29" t="n">
-        <v>1160221.117993379</v>
+        <v>1160211.052004189</v>
       </c>
       <c r="C29" t="n">
-        <v>730000.0165838246</v>
+        <v>728499.5083641879</v>
       </c>
       <c r="D29" t="n">
         <v>19</v>
@@ -2487,7 +2473,7 @@
         <v>270</v>
       </c>
       <c r="F29" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="30">
@@ -2495,10 +2481,10 @@
         <v>28</v>
       </c>
       <c r="B30" t="n">
-        <v>1160476.789595093</v>
+        <v>1160642.761258958</v>
       </c>
       <c r="C30" t="n">
-        <v>729520.9049045217</v>
+        <v>728534.6064685818</v>
       </c>
       <c r="D30" t="n">
         <v>19</v>
@@ -2507,7 +2493,7 @@
         <v>280</v>
       </c>
       <c r="F30" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="31">
@@ -2515,10 +2501,10 @@
         <v>29</v>
       </c>
       <c r="B31" t="n">
-        <v>1160561.445345811</v>
+        <v>1161228.668040063</v>
       </c>
       <c r="C31" t="n">
-        <v>730058.0638181781</v>
+        <v>728173.4793156695</v>
       </c>
       <c r="D31" t="n">
         <v>19</v>
@@ -2527,7 +2513,7 @@
         <v>290</v>
       </c>
       <c r="F31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
@@ -2535,10 +2521,10 @@
         <v>30</v>
       </c>
       <c r="B32" t="n">
-        <v>1160964.510227983</v>
+        <v>1161701.181178588</v>
       </c>
       <c r="C32" t="n">
-        <v>729695.8736891557</v>
+        <v>728391.391087097</v>
       </c>
       <c r="D32" t="n">
         <v>19</v>
@@ -2547,7 +2533,7 @@
         <v>300</v>
       </c>
       <c r="F32" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
@@ -2555,10 +2541,10 @@
         <v>31</v>
       </c>
       <c r="B33" t="n">
-        <v>1160861.534311408</v>
+        <v>1162128.929315304</v>
       </c>
       <c r="C33" t="n">
-        <v>730229.7654407904</v>
+        <v>728688.5740250538</v>
       </c>
       <c r="D33" t="n">
         <v>19</v>
@@ -2567,7 +2553,7 @@
         <v>310</v>
       </c>
       <c r="F33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34">
@@ -2595,10 +2581,10 @@
         <v>33</v>
       </c>
       <c r="B35" t="n">
-        <v>1163657.246433939</v>
+        <v>1162799.898772223</v>
       </c>
       <c r="C35" t="n">
-        <v>728976.5442736079</v>
+        <v>729482.5031677887</v>
       </c>
       <c r="D35" t="n">
         <v>19</v>
@@ -2607,7 +2593,7 @@
         <v>330</v>
       </c>
       <c r="F35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36">
@@ -2735,10 +2721,10 @@
         <v>40</v>
       </c>
       <c r="B42" t="n">
-        <v>1165844.426412606</v>
+        <v>1164548.268319671</v>
       </c>
       <c r="C42" t="n">
-        <v>734213.9050417304</v>
+        <v>733472.3285588899</v>
       </c>
       <c r="D42" t="n">
         <v>19</v>
@@ -2747,7 +2733,7 @@
         <v>30</v>
       </c>
       <c r="F42" t="n">
-        <v>6.5</v>
+        <v>5</v>
       </c>
     </row>
     <row r="43">
@@ -2755,10 +2741,10 @@
         <v>41</v>
       </c>
       <c r="B43" t="n">
-        <v>1165587.627294484</v>
+        <v>1164056.226077507</v>
       </c>
       <c r="C43" t="n">
-        <v>735465.6701534637</v>
+        <v>734189.8722406242</v>
       </c>
       <c r="D43" t="n">
         <v>19</v>
@@ -2767,7 +2753,7 @@
         <v>40</v>
       </c>
       <c r="F43" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="44">
@@ -2935,10 +2921,10 @@
         <v>50</v>
       </c>
       <c r="B52" t="n">
-        <v>1157122.596749579</v>
+        <v>1156742.355473777</v>
       </c>
       <c r="C52" t="n">
-        <v>734776.3013955855</v>
+        <v>735238.6627852177</v>
       </c>
       <c r="D52" t="n">
         <v>19</v>
@@ -2947,7 +2933,7 @@
         <v>130</v>
       </c>
       <c r="F52" t="n">
-        <v>4.9</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="53">
@@ -2955,10 +2941,10 @@
         <v>51</v>
       </c>
       <c r="B53" t="n">
-        <v>1156821.110803118</v>
+        <v>1156064.047860318</v>
       </c>
       <c r="C53" t="n">
-        <v>733916.8896353283</v>
+        <v>734565.0038315067</v>
       </c>
       <c r="D53" t="n">
         <v>19</v>
@@ -2967,7 +2953,7 @@
         <v>140</v>
       </c>
       <c r="F53" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="54">
@@ -3015,10 +3001,10 @@
         <v>54</v>
       </c>
       <c r="B56" t="n">
-        <v>1154362.154373097</v>
+        <v>1154850.962617622</v>
       </c>
       <c r="C56" t="n">
-        <v>732081.9168775</v>
+        <v>731991.7947178755</v>
       </c>
       <c r="D56" t="n">
         <v>19</v>
@@ -3027,7 +3013,7 @@
         <v>170</v>
       </c>
       <c r="F56" t="n">
-        <v>6</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="57">
@@ -3215,10 +3201,10 @@
         <v>64</v>
       </c>
       <c r="B66" t="n">
-        <v>1160207.696806707</v>
+        <v>1160197.631610411</v>
       </c>
       <c r="C66" t="n">
-        <v>727999.3417901163</v>
+        <v>726498.8505219175</v>
       </c>
       <c r="D66" t="n">
         <v>19</v>
@@ -3227,7 +3213,7 @@
         <v>270</v>
       </c>
       <c r="F66" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="67">
@@ -3235,10 +3221,10 @@
         <v>65</v>
       </c>
       <c r="B67" t="n">
-        <v>1160808.731270644</v>
+        <v>1160974.699638183</v>
       </c>
       <c r="C67" t="n">
-        <v>727548.3133127128</v>
+        <v>726562.0254138086</v>
       </c>
       <c r="D67" t="n">
         <v>19</v>
@@ -3247,7 +3233,7 @@
         <v>280</v>
       </c>
       <c r="F67" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="68">
@@ -3255,10 +3241,10 @@
         <v>66</v>
       </c>
       <c r="B68" t="n">
-        <v>1161228.668040063</v>
+        <v>1161895.877459894</v>
       </c>
       <c r="C68" t="n">
-        <v>728173.4793156695</v>
+        <v>726288.9118645781</v>
       </c>
       <c r="D68" t="n">
         <v>19</v>
@@ -3267,7 +3253,7 @@
         <v>290</v>
       </c>
       <c r="F68" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="69">
@@ -3275,10 +3261,10 @@
         <v>67</v>
       </c>
       <c r="B69" t="n">
-        <v>1161946.735885493</v>
+        <v>1162683.393208754</v>
       </c>
       <c r="C69" t="n">
-        <v>727956.564928332</v>
+        <v>726652.0905583026</v>
       </c>
       <c r="D69" t="n">
         <v>19</v>
@@ -3287,7 +3273,7 @@
         <v>300</v>
       </c>
       <c r="F69" t="n">
-        <v>3.5</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70">
@@ -3295,10 +3281,10 @@
         <v>68</v>
       </c>
       <c r="B70" t="n">
-        <v>1162128.929315304</v>
+        <v>1163396.303576563</v>
       </c>
       <c r="C70" t="n">
-        <v>728688.5740250538</v>
+        <v>727147.3862122849</v>
       </c>
       <c r="D70" t="n">
         <v>19</v>
@@ -3307,7 +3293,7 @@
         <v>310</v>
       </c>
       <c r="F70" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="71">
@@ -3335,10 +3321,10 @@
         <v>70</v>
       </c>
       <c r="B72" t="n">
-        <v>1165371.928422857</v>
+        <v>1164514.58964709</v>
       </c>
       <c r="C72" t="n">
-        <v>727964.6178502472</v>
+        <v>728470.5824991141</v>
       </c>
       <c r="D72" t="n">
         <v>19</v>
@@ -3347,7 +3333,7 @@
         <v>330</v>
       </c>
       <c r="F72" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="73">

</xml_diff>